<commit_message>
improved UI from tailwind css to MUI
</commit_message>
<xml_diff>
--- a/backend/app/outputs/audit_report.xlsx
+++ b/backend/app/outputs/audit_report.xlsx
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68</v>
+        <v>92.44</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,7 +605,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>order_id</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -617,13 +617,13 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>customer_name</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -635,7 +635,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4">
@@ -650,10 +650,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5">
@@ -671,13 +671,13 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>country_code</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -689,79 +689,25 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>order_date</t>
+          <t>signup_date</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>datetime64[ns]</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>int64</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>int64</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>payment_mode</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>4</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>